<commit_message>
Add desktop dev stories page
</commit_message>
<xml_diff>
--- a/docs/assets/exhibit-asset-tracker.xlsx
+++ b/docs/assets/exhibit-asset-tracker.xlsx
@@ -1,18 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="legend" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="scene_assets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="exhibits" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="gallery_nodes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="legend" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="scene_assets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="exhibits" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="gallery_nodes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'legend'!$A$1:$B$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'scene_assets'!$A$1:$E$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'exhibits'!$A$1:$U$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'gallery_nodes'!$A$1:$E$19</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -20,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,16 +33,25 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F2937"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +59,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D1D5DB"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -125,6 +159,75 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="legend_table" displayName="legend_table" ref="A1:B13" headerRowCount="1">
+  <autoFilter ref="A1:B13"/>
+  <tableColumns count="2">
+    <tableColumn id="1" name="字段/值"/>
+    <tableColumn id="2" name="说明"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="scene_assets_table" displayName="scene_assets_table" ref="A1:E4" headerRowCount="1">
+  <autoFilter ref="A1:E4"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="asset_key"/>
+    <tableColumn id="2" name="path"/>
+    <tableColumn id="3" name="exists"/>
+    <tableColumn id="4" name="status"/>
+    <tableColumn id="5" name="notes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="exhibits_table" displayName="exhibits_table" ref="A1:U3" headerRowCount="1">
+  <autoFilter ref="A1:U3"/>
+  <tableColumns count="21">
+    <tableColumn id="1" name="exhibitId"/>
+    <tableColumn id="2" name="sceneObjectName"/>
+    <tableColumn id="3" name="type"/>
+    <tableColumn id="4" name="zone"/>
+    <tableColumn id="5" name="status"/>
+    <tableColumn id="6" name="in_gallery_main"/>
+    <tableColumn id="7" name="folder_path"/>
+    <tableColumn id="8" name="focus_glb_file"/>
+    <tableColumn id="9" name="focus_glb_exists"/>
+    <tableColumn id="10" name="audio_file"/>
+    <tableColumn id="11" name="audio_exists"/>
+    <tableColumn id="12" name="video_file"/>
+    <tableColumn id="13" name="video_exists"/>
+    <tableColumn id="14" name="image_file"/>
+    <tableColumn id="15" name="image_exists"/>
+    <tableColumn id="16" name="in_manifest"/>
+    <tableColumn id="17" name="manifest_buttons"/>
+    <tableColumn id="18" name="focusGlbUrl"/>
+    <tableColumn id="19" name="notes"/>
+    <tableColumn id="20" name="last_updated"/>
+    <tableColumn id="21" name="owner"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="gallery_nodes_table" displayName="gallery_nodes_table" ref="A1:E19" headerRowCount="1">
+  <autoFilter ref="A1:E19"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="node_name"/>
+    <tableColumn id="2" name="node_type"/>
+    <tableColumn id="3" name="y_range"/>
+    <tableColumn id="4" name="code_binding"/>
+    <tableColumn id="5" name="notes"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -418,165 +521,173 @@
   </sheetPr>
   <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>﻿字段/值</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>字段/值</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>status: 待制作</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>尚未开始建模或导出</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>status: 制作中</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>DCC 进行中或待入库</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>status: 已入库</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>文件已放入 public 对应路径</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>status: 需调整</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>已入库但命名/尺度/manifest 需改</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>status: 已验收</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>联调通过</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Y / N</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>文件或绑定是否就绪；入库后改为 Y</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>exhibitId</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>与 manifest.json 的 exhibitId 一致</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>sceneObjectName</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>gallery_main 内 hit mesh，规则 exhibit_&lt;exhibitId&gt;</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>focus_glb_file</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>位于 folder_path 下，建议 focus_&lt;exhibitId&gt;.glb</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>in_manifest</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>manifest.json 是否已有该条目（代码可先配好为 Y）</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>维护顺序</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>新增行 → 建目录 → 做 glb/媒体 → 更新 manifest → 改 Y</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>对照文档</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>docs/gallery-mesh-naming.md / docs/asset-manifest.md / exhibit-asset-tracker-gallery_nodes.csv</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:B13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -588,117 +699,128 @@
   </sheetPr>
   <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>﻿asset_key</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>asset_key</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>path</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>exists</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>gallery_main</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>models/gallery_main.glb</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>已入库</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-06-01 覆写：节点未变；spawn_player_main XZ=(11.576,-8.13) Empty Y≈3 仅参考，运行时 bodyY=0.92</t>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-02 更新：+COL_sidetable_1；spawn XZ≈(5.034,-0.865)；17 mesh；可见≈17.7k tris</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>bgm_architecture</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>audio/bgm_architecture.mp3</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>待制作</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>进入 SPACE 后 architecture 分区 BGM</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>wall_art</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>media/art_01.jpg</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>可选</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>北墙代码画框贴图（ENABLE_GALLERY_WALL_ART=false）</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -708,205 +830,307 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U2"/>
+  <dimension ref="A1:U3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="30" customWidth="1" min="17" max="17"/>
+    <col width="41" customWidth="1" min="18" max="18"/>
+    <col width="36" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>﻿exhibitId</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>exhibitId</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>sceneObjectName</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>zone</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>in_gallery_main</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>folder_path</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>focus_glb_file</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>focus_glb_exists</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>audio_file</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>audio_exists</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>video_file</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>video_exists</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>image_file</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>image_exists</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>in_manifest</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>manifest_buttons</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>focusGlbUrl</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>last_updated</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>owner</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>demo_box</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>exhibit_demo_box</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>audio</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>architecture</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>制作中</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>exhibits/demo_box/</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>focus_demo_box.glb</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>demo.mp3</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>demo_box.mp3</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>btn_play, btn_pause, btn_end</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>/exhibits/demo_box/focus_demo_box.glb</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="S2" s="2" t="inlineStr">
         <is>
           <t>gallery_main 已同步 2026-06-01 覆写</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="T2" s="2" t="inlineStr">
         <is>
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr"/>
+      <c r="U2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>demo_bass</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>exhibit_demo_bass</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>model3d</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>architecture</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>制作中</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>exhibits/demo_bass/</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>focus_demo_bass.glb</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr"/>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr"/>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>/exhibits/demo_bass/focus_demo_bass.glb</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>gallery_main exhibit_demo_bass 已同步</t>
+        </is>
+      </c>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:U3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -916,465 +1140,530 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>node_name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>node_type</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>y_range</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>code_binding</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>COL_ground</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>mesh</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>-0.99~0.00</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>GalleryFloorCollider + walkable spawn</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>地板碰撞（优先读取此名）</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>COL_inner_1</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>mesh</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>2.00~4.00</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>ColColliders cuboid</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>内墙碰撞</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>COL_inner_2</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>mesh</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>0.00~1.00</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>ColColliders cuboid</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>内墙碰撞</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>COL_inner_3</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>mesh</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>0.00~4.00</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>ColColliders cuboid</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>内墙碰撞</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>COL_outer_1</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>mesh</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>0.00~4.00</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>ColColliders trimesh (double-sided)</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>外墙碰撞</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>COL_platform_1</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>mesh</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>0.00~0.50</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>ColColliders trimesh + GalleryFloorCollider cutout</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>平台含台阶</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>COL_sidetable_1</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>mesh</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>0.00~0.77</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>ColColliders trimesh</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>外墙碰撞（法线需朝室内）</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>COL_platform_1</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>边桌碰撞（GLB 2026-06-05 已入库）</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>spawn_player_main</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>empty</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>resolveGallerySpawn</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>出生 Empty XZ≈(5.034,-0.865)；Y 由脚下地面算 bodyY≈0.92</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>exhibit_demo_box</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>mesh</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>0.77~0.98</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>bindExhibitIds → demo_box</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>交互 hit mesh</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>exhibit_demo_bass</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>mesh</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>0.89~0.96</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>bindExhibitIds → demo_bass</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>贝司交互 hit mesh</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>prop_sidetable_1</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>mesh</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>0.00~0.77</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>视觉 only</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>装饰道具，无碰撞</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>struct_ground</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>mesh</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>-0.99~0.00</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>视觉</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>地面对应 struct_ground</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>struct_inner_1</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>mesh</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>2.00~4.00</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>视觉</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>内墙视觉</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>struct_inner_2</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>mesh</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>0.00~1.00</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>视觉</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>内墙视觉</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>struct_inner_3</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>mesh</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>0.00~4.00</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>视觉</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>内墙视觉</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>struct_outer_1</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>mesh</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>0.00~4.00</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>视觉</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>外墙视觉</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>struct_ceiling_1</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>mesh</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>4.00~4.00</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>视觉</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>天花</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>struct_platform_1</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>mesh</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>0.00~0.50</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>walkable spawn only</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>平台（无独立物理地板）</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>spawn_player_main</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>resolveGallerySpawn</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>出生 Empty；代码读 XZ，Y 由 COL_ground 顶面算（≈0.92），忽略 Empty 的 Y</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>exhibit_demo_box</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>mesh</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>0.77~0.98</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>bindExhibitIds → demo_box</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>交互 hit mesh</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>prop_sidetable_1</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>mesh</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>0.00~0.77</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>视觉 only</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>装饰道具，无碰撞</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>struct_ground</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>mesh</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>-0.99~0.00</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>视觉</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>地面对应 struct_ground</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>struct_inner_1</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>mesh</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>2.00~4.00</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>视觉</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>内墙视觉</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>struct_inner_2</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>mesh</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>0.00~1.00</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>视觉</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>内墙视觉</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>struct_inner_3</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>mesh</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>0.00~4.00</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>视觉</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>内墙视觉</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>struct_outer_1</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>mesh</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>0.00~4.00</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>视觉</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>外墙视觉</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>struct_ceiling_1</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>mesh</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>4.00~4.00</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>视觉</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>天花</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>struct_platform_1</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>mesh</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>0.00~0.50</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>视觉</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>平台视觉</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E19"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: update space experience assets
</commit_message>
<xml_diff>
--- a/docs/assets/exhibit-asset-tracker.xlsx
+++ b/docs/assets/exhibit-asset-tracker.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -36,6 +36,9 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -77,7 +80,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -85,6 +88,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -523,160 +527,160 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>字段/值</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>说明</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>status: 待制作</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>尚未开始建模或导出</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>status: 制作中</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>DCC 进行中或待入库</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>status: 已入库</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>文件已放入 public 对应路径</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>status: 需调整</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>已入库但命名/尺度/manifest 需改</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>status: 已验收</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>联调通过</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Y / N</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>文件或绑定是否就绪；入库后改为 Y</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>exhibitId</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>与 manifest.json 的 exhibitId 一致</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>sceneObjectName</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>gallery_main 内 hit mesh，规则 exhibit_&lt;exhibitId&gt;</t>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>space_main 内 hit mesh，规则 exhibit_&lt;exhibitId&gt;</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>focus_glb_file</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>位于 folder_path 下，建议 focus_&lt;exhibitId&gt;.glb</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>in_manifest</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>manifest.json 是否已有该条目（代码可先配好为 Y）</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>维护顺序</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>新增行 → 建目录 → 做 glb/媒体 → 更新 manifest → 改 Y</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>对照文档</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>docs/gallery-mesh-naming.md / docs/asset-manifest.md / exhibit-asset-tracker-gallery_nodes.csv</t>
         </is>
@@ -697,119 +701,146 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>asset_key</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>path</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>exists</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>gallery_main</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>space_main</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>models/space_main.glb</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>已入库</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-06-14 处理：12 个 COL_floor_*、2 个 bulb_*、spawn_player_main；92 mesh；约 8.4k tris；无 required glTF extensions</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>gallery_main_demo</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>models/gallery_main.glb</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>已入库</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-02 更新：+COL_sidetable_1；spawn XZ≈(5.034,-0.865)；17 mesh；可见≈17.7k tris</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>历史 demo</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>gallery_main 仅保留测试 / 历史对照，不再作为生产展厅空间</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>bgm_architecture</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>audio/bgm_architecture.mp3</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>待制作</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>进入 SPACE 后 architecture 分区 BGM</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
         <is>
           <t>wall_art</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>media/art_01.jpg</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>可选</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>北墙代码画框贴图（ENABLE_GALLERY_WALL_ART=false）</t>
         </is>
@@ -838,7 +869,7 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
@@ -851,279 +882,279 @@
     <col width="13" customWidth="1" min="16" max="16"/>
     <col width="30" customWidth="1" min="17" max="17"/>
     <col width="41" customWidth="1" min="18" max="18"/>
-    <col width="36" customWidth="1" min="19" max="19"/>
+    <col width="48" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
     <col width="10" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>exhibitId</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>sceneObjectName</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>type</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>zone</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>in_gallery_main</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>in_space_main</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>folder_path</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>focus_glb_file</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>focus_glb_exists</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>audio_file</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>audio_exists</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>video_file</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>video_exists</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>image_file</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>image_exists</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>in_manifest</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>manifest_buttons</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" s="3" t="inlineStr">
         <is>
           <t>focusGlbUrl</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" s="3" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" s="3" t="inlineStr">
         <is>
           <t>last_updated</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" s="3" t="inlineStr">
         <is>
           <t>owner</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>demo_box</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>exhibit_demo_box</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>audio</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>architecture</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>制作中</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>exhibits/demo_box/</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>focus_demo_box.glb</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>exhibits/demo_box/</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>focus_demo_box.glb</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>demo_box.mp3</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
-        <is>
-          <t>demo_box.mp3</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>btn_play, btn_pause, btn_end</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>/exhibits/demo_box/focus_demo_box.glb</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>space_main 当前未放置 exhibit_* hit mesh；gallery_main 仅保留历史 demo</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>demo_bass</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>exhibit_demo_bass</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>model3d</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>architecture</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>制作中</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr"/>
-      <c r="N2" s="2" t="inlineStr"/>
-      <c r="O2" s="2" t="inlineStr"/>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>exhibits/demo_bass/</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>focus_demo_bass.glb</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr">
-        <is>
-          <t>btn_play, btn_pause, btn_end</t>
-        </is>
-      </c>
-      <c r="R2" s="2" t="inlineStr">
-        <is>
-          <t>/exhibits/demo_box/focus_demo_box.glb</t>
-        </is>
-      </c>
-      <c r="S2" s="2" t="inlineStr">
-        <is>
-          <t>gallery_main 已同步 2026-06-01 覆写</t>
-        </is>
-      </c>
-      <c r="T2" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-01</t>
-        </is>
-      </c>
-      <c r="U2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>demo_bass</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>exhibit_demo_bass</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>model3d</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>architecture</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>制作中</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>exhibits/demo_bass/</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>focus_demo_bass.glb</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr"/>
-      <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="inlineStr"/>
-      <c r="N3" s="2" t="inlineStr"/>
-      <c r="O3" s="2" t="inlineStr"/>
-      <c r="P3" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="Q3" s="2" t="inlineStr"/>
-      <c r="R3" s="2" t="inlineStr">
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
         <is>
           <t>/exhibits/demo_bass/focus_demo_bass.glb</t>
         </is>
       </c>
-      <c r="S3" s="2" t="inlineStr">
-        <is>
-          <t>gallery_main exhibit_demo_bass 已同步</t>
-        </is>
-      </c>
-      <c r="T3" s="2" t="inlineStr">
-        <is>
-          <t>2026-06-07</t>
-        </is>
-      </c>
-      <c r="U3" s="2" t="inlineStr"/>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>space_main 当前未放置 exhibit_* hit mesh；gallery_main 仅保留历史 demo</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:U3"/>

</xml_diff>